<commit_message>
feat(seeding): enhance store schema with home service and pickup/delivery zones
</commit_message>
<xml_diff>
--- a/data/Data Store.xlsx
+++ b/data/Data Store.xlsx
@@ -28,7 +28,7 @@
     <t>is_default_store</t>
   </si>
   <si>
-    <t>is_pick_up_available</t>
+    <t>is_pickup_delivery_available</t>
   </si>
   <si>
     <t>location</t>
@@ -43,7 +43,7 @@
     <t>capacity</t>
   </si>
   <si>
-    <t>zones</t>
+    <t>home_service_zones</t>
   </si>
   <si>
     <t>is_active</t>
@@ -106,7 +106,7 @@
     <t>travel_time_minutes</t>
   </si>
   <si>
-    <t>travel_fee</t>
+    <t>price</t>
   </si>
   <si>
     <t>STR001</t>
@@ -300,43 +300,46 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -555,8 +558,10 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
+    <col customWidth="1" min="4" max="4" width="15.75"/>
     <col customWidth="1" min="5" max="5" width="21.63"/>
     <col customWidth="1" min="6" max="6" width="18.63"/>
+    <col customWidth="1" min="7" max="7" width="16.75"/>
     <col customWidth="1" min="18" max="18" width="42.0"/>
     <col customWidth="1" min="20" max="21" width="26.0"/>
     <col customWidth="1" min="24" max="24" width="15.0"/>
@@ -699,7 +704,7 @@
         <v>34</v>
       </c>
       <c r="E3" s="8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="8" t="b">
         <v>1</v>
@@ -713,13 +718,13 @@
       <c r="I3" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="J3" s="7">
+      <c r="J3" s="1">
         <v>60284.0</v>
       </c>
-      <c r="K3" s="7">
+      <c r="K3" s="1">
         <v>-7.275615</v>
       </c>
-      <c r="L3" s="7">
+      <c r="L3" s="1">
         <v>112.782414</v>
       </c>
       <c r="M3" s="7"/>
@@ -737,69 +742,69 @@
         <v>41</v>
       </c>
       <c r="S3" s="7"/>
-      <c r="T3" s="7">
+      <c r="T3" s="1">
         <v>1620.0</v>
       </c>
-      <c r="U3" s="7">
+      <c r="U3" s="1">
         <v>120.0</v>
       </c>
       <c r="V3" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="W3" s="12">
+      <c r="W3" s="6">
         <v>0.0</v>
       </c>
-      <c r="X3" s="12">
+      <c r="X3" s="6">
         <v>5.0</v>
       </c>
-      <c r="Y3" s="12">
+      <c r="Y3" s="6">
         <v>0.0</v>
       </c>
-      <c r="Z3" s="12">
+      <c r="Z3" s="13">
         <v>10000.0</v>
       </c>
-      <c r="AA3" s="12" t="b">
+      <c r="AA3" s="6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="14"/>
+      <c r="S4" s="14"/>
+      <c r="T4" s="14"/>
+      <c r="U4" s="14"/>
       <c r="V4" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="W4" s="12">
+      <c r="W4" s="6">
         <v>6.0</v>
       </c>
-      <c r="X4" s="12">
+      <c r="X4" s="6">
         <v>10.0</v>
       </c>
-      <c r="Y4" s="12">
+      <c r="Y4" s="6">
         <v>0.0</v>
       </c>
-      <c r="Z4" s="12">
+      <c r="Z4" s="13">
         <v>20000.0</v>
       </c>
-      <c r="AA4" s="12" t="b">
+      <c r="AA4" s="6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -828,19 +833,19 @@
       <c r="V5" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W5" s="12">
+      <c r="W5" s="6">
         <v>11.0</v>
       </c>
-      <c r="X5" s="12">
+      <c r="X5" s="6">
         <v>30.0</v>
       </c>
-      <c r="Y5" s="12">
+      <c r="Y5" s="6">
         <v>0.0</v>
       </c>
-      <c r="Z5" s="12">
+      <c r="Z5" s="13">
         <v>40000.0</v>
       </c>
-      <c r="AA5" s="12" t="b">
+      <c r="AA5" s="6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -857,10 +862,10 @@
       <c r="D6" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14" t="b">
+      <c r="E6" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="15" t="b">
         <v>1</v>
       </c>
       <c r="G6" s="7" t="s">
@@ -872,13 +877,13 @@
       <c r="I6" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="1">
         <v>60213.0</v>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="1">
         <v>-7.312938</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="1">
         <v>112.768221</v>
       </c>
       <c r="M6" s="7"/>
@@ -896,69 +901,69 @@
         <v>41</v>
       </c>
       <c r="S6" s="7"/>
-      <c r="T6" s="7">
+      <c r="T6" s="1">
         <v>1620.0</v>
       </c>
-      <c r="U6" s="7">
+      <c r="U6" s="1">
         <v>120.0</v>
       </c>
       <c r="V6" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="W6" s="12">
+      <c r="W6" s="6">
         <v>0.0</v>
       </c>
-      <c r="X6" s="12">
+      <c r="X6" s="6">
         <v>5.0</v>
       </c>
-      <c r="Y6" s="12">
+      <c r="Y6" s="6">
         <v>0.0</v>
       </c>
-      <c r="Z6" s="12">
+      <c r="Z6" s="13">
         <v>10000.0</v>
       </c>
-      <c r="AA6" s="12" t="b">
+      <c r="AA6" s="6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="13"/>
-      <c r="S7" s="13"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="13"/>
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
       <c r="V7" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="W7" s="12">
+      <c r="W7" s="6">
         <v>6.0</v>
       </c>
-      <c r="X7" s="12">
+      <c r="X7" s="6">
         <v>10.0</v>
       </c>
-      <c r="Y7" s="12">
+      <c r="Y7" s="6">
         <v>0.0</v>
       </c>
-      <c r="Z7" s="12">
+      <c r="Z7" s="13">
         <v>20000.0</v>
       </c>
-      <c r="AA7" s="12" t="b">
+      <c r="AA7" s="6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -987,19 +992,19 @@
       <c r="V8" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="W8" s="12">
+      <c r="W8" s="6">
         <v>11.0</v>
       </c>
-      <c r="X8" s="12">
+      <c r="X8" s="6">
         <v>30.0</v>
       </c>
-      <c r="Y8" s="12">
+      <c r="Y8" s="6">
         <v>0.0</v>
       </c>
-      <c r="Z8" s="12">
+      <c r="Z8" s="13">
         <v>40000.0</v>
       </c>
-      <c r="AA8" s="12" t="b">
+      <c r="AA8" s="6" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>